<commit_message>
Redondeo desde lo que muestra la lamina, fila Nacional en XLSX de Ingresos, reintento de payloads y aviso de anio sin dato en correlaciones
</commit_message>
<xml_diff>
--- a/output/graficos_regionales/plot_i_ingr_a_2018_antofagasta.xlsx
+++ b/output/graficos_regionales/plot_i_ingr_a_2018_antofagasta.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve">indicador</t>
   </si>
@@ -90,6 +90,9 @@
     <t xml:space="preserve">Antofagasta</t>
   </si>
   <si>
+    <t xml:space="preserve">Nacional</t>
+  </si>
+  <si>
     <t xml:space="preserve">Campo</t>
   </si>
   <si>
@@ -99,7 +102,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-25 21:27</t>
+    <t xml:space="preserve">2026-10-03 19:31</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -825,7 +828,9 @@
       <c r="A18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="2"/>
+      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="n">
         <v>2018</v>
@@ -854,58 +859,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_regionales)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales/plot_i_ingr_a_2018_antofagasta.xlsx
+++ b/output/graficos_regionales/plot_i_ingr_a_2018_antofagasta.xlsx
@@ -102,7 +102,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-03 19:31</t>
+    <t xml:space="preserve">2026-10-05 01:57</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -762,7 +762,7 @@
         <v>2018</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>857521.62</v>
+        <v>857521.63</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -781,7 +781,7 @@
         <v>2018</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>898577.12</v>
+        <v>898577.13</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -836,7 +836,7 @@
         <v>2018</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>812081.12</v>
+        <v>812081.13</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>

</xml_diff>